<commit_message>
Regenerate Excel test case document after session refresh
Re-ran the full suite (37 passed, 0 failed, 3 skipped) against a
freshly re-authenticated session to confirm the earlier session-expiry
failures were not application defects.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SuAphcog1d9DyVnHBUw5kX
</commit_message>
<xml_diff>
--- a/reports/Aperion-Test-Cases.xlsx
+++ b/reports/Aperion-Test-Cases.xlsx
@@ -17,7 +17,7 @@
     <t>Aperion Health - Wellness / Advisor Portal - Test Case Document</t>
   </si>
   <si>
-    <t>Generated: 2026-09-02     |     Total Test Cases: 158     |     Automated: 39     |     Manual: 119     |     Pass: 155     |     Fail: 1</t>
+    <t>Generated: 2026-09-03     |     Total Test Cases: 158     |     Automated: 39     |     Manual: 119     |     Pass: 155     |     Fail: 1</t>
   </si>
   <si>
     <t>Manual cases are imported from the team sheet (npm run import). Automated cases are filled in by the Playwright suite - where an automated test reuses a case ID, its run result replaces the manual Status and Actual Result. Status is a dropdown; colours follow the value.</t>
@@ -3231,13 +3231,13 @@
   <si>
     <t xml:space="preserve">1. Pre-flight refresh tops up aperion_token via /api/v1/auth/refresh.
 2. Open the protected route (SMOKE_ROUTE, default /wellness/dashboard) with the saved storage state.
-3. Check the landing URL and read aperion_token from localStorage.</t>
+3. Check the landing URL, the rendered content and aperion_token in localStorage.</t>
   </si>
   <si>
     <t>auth/auth.json (localStorage: aperion_token, aperion_refresh_token)</t>
   </si>
   <si>
-    <t>The dashboard loads without redirecting to /login, and a non-empty aperion_token is present in localStorage.</t>
+    <t>The dashboard loads without redirecting to /login, the logged-out marketing/OTP screen is not shown, and a non-empty aperion_token is present in localStorage.</t>
   </si>
   <si>
     <t>As expected.</t>

</xml_diff>